<commit_message>
feat(pivot): evaluate authored relative-period and top-N flavour filters
- decode <filter type="thisMonth"> and its day/month/quarter/year/year-to-date siblings into a new AuthoredPeriodFilter list
- record the top-N basis (count/percent/sum) that the identically shaped <top10> element cannot distinguish
- resolve a period into an inclusive serial window against the clock reading, read once per evaluation and threaded through the new PivotFilterEnv
- keep the descending-ranked leaves until the running total first reaches the target for the percent and sum top-N flavours
- week windows and the recurring M1..M12 / Q1..Q4 selectors stay undecoded
- pin the percent and sum behaviour against the excel-authored fixture tests/fixtures/excel/pivot_value_date_filters.xlsx (two new sheets), which formulon matches, and update tests/divergence.yaml accordingly
</commit_message>
<xml_diff>
--- a/tests/fixtures/excel/pivot_value_date_filters.xlsx
+++ b/tests/fixtures/excel/pivot_value_date_filters.xlsx
@@ -5,23 +5,25 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/libraz/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/libraz/Projects/formulon/tests/fixtures/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{62DC7F12-20F4-DA45-8A34-E81A1F598607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{815D6D77-C832-1D42-9772-7E70E65A82BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35020" yWindow="7880" windowWidth="28300" windowHeight="17360" activeTab="3" xr2:uid="{0682156C-DB83-E945-B13C-A138789C4A08}"/>
+    <workbookView xWindow="35020" yWindow="7880" windowWidth="28300" windowHeight="17360" activeTab="5" xr2:uid="{0682156C-DB83-E945-B13C-A138789C4A08}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
     <sheet name="Sheet4" sheetId="4" r:id="rId3"/>
     <sheet name="Sheet5" sheetId="5" r:id="rId4"/>
-    <sheet name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet name="Sheet6" sheetId="6" r:id="rId5"/>
+    <sheet name="Sheet7" sheetId="7" r:id="rId6"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId7"/>
   </sheets>
   <calcPr calcId="181029"/>
   <pivotCaches>
-    <pivotCache cacheId="9" r:id="rId6"/>
+    <pivotCache cacheId="12" r:id="rId8"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -46,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="13">
   <si>
     <t>North</t>
   </si>
@@ -139,9 +141,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1">
       <alignment vertical="center"/>
     </xf>
@@ -150,6 +149,9 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -272,7 +274,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CC67DE83-3E0F-7A4E-AF68-3135DB691947}" name="ピボットテーブル1" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CC67DE83-3E0F-7A4E-AF68-3135DB691947}" name="ピボットテーブル1" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" showAll="0" measureFilter="1">
@@ -342,7 +344,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0B06916C-3AA8-274F-A2B3-A2F4613D3C4C}" name="ピボットテーブル2" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0B06916C-3AA8-274F-A2B3-A2F4613D3C4C}" name="ピボットテーブル2" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" showAll="0" measureFilter="1">
@@ -417,7 +419,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F4FE278B-4D0E-964C-BAFD-D06DC8B88100}" name="ピボットテーブル3" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F4FE278B-4D0E-964C-BAFD-D06DC8B88100}" name="ピボットテーブル3" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" showAll="0" measureFilter="1">
@@ -505,7 +507,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{54CF710F-D841-8B40-8DF2-8F1267AE6691}" name="ピボットテーブル4" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{54CF710F-D841-8B40-8DF2-8F1267AE6691}" name="ピボットテーブル4" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField showAll="0"/>
@@ -563,6 +565,119 @@
             <customFilter operator="greaterThanOrEqual" val="45292"/>
             <customFilter operator="lessThanOrEqual" val="45382"/>
           </customFilters>
+        </filterColumn>
+      </autoFilter>
+    </filter>
+  </filters>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D2B6EBD6-CEFF-2D43-988A-FB054E8E8FC7}" name="ピボットテーブル5" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="4">
+    <pivotField axis="axisRow" showAll="0" measureFilter="1">
+      <items count="5">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="合計 / Amt" fld="3" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <filters count="1">
+    <filter fld="0" type="percent" evalOrder="-1" id="2" iMeasureFld="0">
+      <autoFilter ref="A1">
+        <filterColumn colId="0">
+          <top10 percent="1" val="70" filterVal="70"/>
+        </filterColumn>
+      </autoFilter>
+    </filter>
+  </filters>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7C19155A-D53B-DC49-8671-353DCD7CE588}" name="ピボットテーブル6" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:B5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="4">
+    <pivotField axis="axisRow" showAll="0" measureFilter="1">
+      <items count="5">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="2">
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="合計 / Amt" fld="3" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <filters count="1">
+    <filter fld="0" type="sum" evalOrder="-1" id="4" iMeasureFld="0">
+      <autoFilter ref="A1">
+        <filterColumn colId="0">
+          <top10 val="100" filterVal="100"/>
         </filterColumn>
       </autoFilter>
     </filter>
@@ -903,7 +1018,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B3" t="s">
@@ -911,26 +1026,26 @@
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4">
         <v>500</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5">
         <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6">
         <v>675</v>
       </c>
     </row>
@@ -949,7 +1064,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B3" t="s">
@@ -957,34 +1072,34 @@
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4">
         <v>150</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5">
         <v>500</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6">
         <v>175</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7">
         <v>825</v>
       </c>
     </row>
@@ -1004,7 +1119,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B3" t="s">
@@ -1012,34 +1127,34 @@
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4">
         <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5">
         <v>150</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6">
         <v>175</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7">
         <v>425</v>
       </c>
     </row>
@@ -1058,7 +1173,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B3" t="s">
@@ -1066,50 +1181,50 @@
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="5">
+      <c r="A4" s="4">
         <v>45306</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4">
         <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="5">
+      <c r="A5" s="4">
         <v>45316</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5">
         <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="5">
+      <c r="A6" s="4">
         <v>45330</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6">
         <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="5">
+      <c r="A7" s="4">
         <v>45342</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7">
         <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="5">
+      <c r="A8" s="4">
         <v>45361</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8">
         <v>200</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9">
         <v>580</v>
       </c>
     </row>
@@ -1120,6 +1235,90 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BB02E7D-A7C8-A14B-B473-13642731F247}">
+  <dimension ref="A3:B6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
+  <cols>
+    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:2">
+      <c r="A3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="5">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="5">
+        <v>675</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A0C7AA1-1350-C64F-9816-7AADB36A0530}">
+  <dimension ref="A3:B5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
+  <cols>
+    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:2">
+      <c r="A3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="5">
+        <v>500</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D90E86F0-D4F9-5440-8F3D-7AAA371A580E}">
   <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>

</xml_diff>

<commit_message>
test(pivot): pin top-n percent against the accumulated total
- rebuild tests/fixtures/excel/pivot_value_date_filters.xlsx with a Top-N
  "50 percent" pivot on Region; the source table now sits on Sheet1
- excel's cached render of that pivot is the single South row: 50 percent
  of the 925 measure total is 462.5, which South clears alone, whereas a
  share of the 4-item count would have kept West as well
- note on the existing 70 percent case that it cannot separate the two
  readings, since both keep exactly South and West there
- clarify the percent branch of build_running_total_keep in
  src/pivot/filter_engine.cpp to point at the fixture; comment only
</commit_message>
<xml_diff>
--- a/tests/fixtures/excel/pivot_value_date_filters.xlsx
+++ b/tests/fixtures/excel/pivot_value_date_filters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/libraz/Projects/formulon/tests/fixtures/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{815D6D77-C832-1D42-9772-7E70E65A82BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D262560-042F-BA41-8FBC-833383778941}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35020" yWindow="7880" windowWidth="28300" windowHeight="17360" activeTab="5" xr2:uid="{0682156C-DB83-E945-B13C-A138789C4A08}"/>
+    <workbookView xWindow="35020" yWindow="7880" windowWidth="28300" windowHeight="17360" activeTab="6" xr2:uid="{0682156C-DB83-E945-B13C-A138789C4A08}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -19,11 +19,12 @@
     <sheet name="Sheet5" sheetId="5" r:id="rId4"/>
     <sheet name="Sheet6" sheetId="6" r:id="rId5"/>
     <sheet name="Sheet7" sheetId="7" r:id="rId6"/>
-    <sheet name="Sheet1" sheetId="1" r:id="rId7"/>
+    <sheet name="Sheet8" sheetId="8" r:id="rId7"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId8"/>
   </sheets>
   <calcPr calcId="181029"/>
   <pivotCaches>
-    <pivotCache cacheId="12" r:id="rId8"/>
+    <pivotCache cacheId="8" r:id="rId9"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="13">
   <si>
     <t>North</t>
   </si>
@@ -274,7 +275,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CC67DE83-3E0F-7A4E-AF68-3135DB691947}" name="ピボットテーブル1" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CC67DE83-3E0F-7A4E-AF68-3135DB691947}" name="ピボットテーブル1" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" showAll="0" measureFilter="1">
@@ -344,7 +345,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0B06916C-3AA8-274F-A2B3-A2F4613D3C4C}" name="ピボットテーブル2" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0B06916C-3AA8-274F-A2B3-A2F4613D3C4C}" name="ピボットテーブル2" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" showAll="0" measureFilter="1">
@@ -419,7 +420,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F4FE278B-4D0E-964C-BAFD-D06DC8B88100}" name="ピボットテーブル3" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F4FE278B-4D0E-964C-BAFD-D06DC8B88100}" name="ピボットテーブル3" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" showAll="0" measureFilter="1">
@@ -507,7 +508,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{54CF710F-D841-8B40-8DF2-8F1267AE6691}" name="ピボットテーブル4" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{54CF710F-D841-8B40-8DF2-8F1267AE6691}" name="ピボットテーブル4" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField showAll="0"/>
@@ -581,7 +582,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D2B6EBD6-CEFF-2D43-988A-FB054E8E8FC7}" name="ピボットテーブル5" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D2B6EBD6-CEFF-2D43-988A-FB054E8E8FC7}" name="ピボットテーブル5" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" showAll="0" measureFilter="1">
@@ -639,7 +640,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7C19155A-D53B-DC49-8671-353DCD7CE588}" name="ピボットテーブル6" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7C19155A-D53B-DC49-8671-353DCD7CE588}" name="ピボットテーブル6" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" showAll="0" measureFilter="1">
@@ -678,6 +679,61 @@
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <top10 val="100" filterVal="100"/>
+        </filterColumn>
+      </autoFilter>
+    </filter>
+  </filters>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{13E2F45A-A7D0-5547-8567-EA32CC1C0B97}" name="ピボットテーブル1" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="値" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:B5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="4">
+    <pivotField axis="axisRow" showAll="0" measureFilter="1">
+      <items count="5">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="2">
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="合計 / Amt" fld="3" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <filters count="1">
+    <filter fld="0" type="percent" evalOrder="-1" id="2" iMeasureFld="0">
+      <autoFilter ref="A1">
+        <filterColumn colId="0">
+          <top10 percent="1" val="50" filterVal="50"/>
         </filterColumn>
       </autoFilter>
     </filter>
@@ -1254,7 +1310,7 @@
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4">
         <v>500</v>
       </c>
     </row>
@@ -1262,7 +1318,7 @@
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5">
         <v>175</v>
       </c>
     </row>
@@ -1270,7 +1326,7 @@
       <c r="A6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6">
         <v>675</v>
       </c>
     </row>
@@ -1300,7 +1356,7 @@
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4">
         <v>500</v>
       </c>
     </row>
@@ -1308,7 +1364,7 @@
       <c r="A5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5">
         <v>500</v>
       </c>
     </row>
@@ -1319,6 +1375,44 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB228990-150E-DF4D-9B59-C13CA17A0521}">
+  <dimension ref="A3:B5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
+  <cols>
+    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:2">
+      <c r="A3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="5">
+        <v>500</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D90E86F0-D4F9-5440-8F3D-7AAA371A580E}">
   <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>

</xml_diff>